<commit_message>
reliability eval first results
</commit_message>
<xml_diff>
--- a/results/reliability_eval/unified_scores_table.xlsx
+++ b/results/reliability_eval/unified_scores_table.xlsx
@@ -535,17 +535,17 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>P178</t>
+          <t>beam</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>tokens</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -589,17 +589,17 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>P101</t>
+          <t>beam</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>tokens</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -643,17 +643,17 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>P1376</t>
+          <t>beam</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>tokens</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -697,17 +697,17 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>P103</t>
+          <t>beam</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>tokens</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -751,17 +751,17 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>P27</t>
+          <t>beam</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>tokens</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -805,17 +805,17 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>P108</t>
+          <t>beam</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>tokens</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -859,17 +859,17 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>P17</t>
+          <t>beam</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>tokens</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -913,17 +913,17 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>P176</t>
+          <t>beam</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>tokens</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -967,17 +967,17 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>P19</t>
+          <t>beam</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>tokens</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1021,17 +1021,17 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>P264</t>
+          <t>beam</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>tokens</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1075,17 +1075,17 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>P1412</t>
+          <t>beam</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>tokens</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1129,17 +1129,17 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>10</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>tokens</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>temp</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1183,17 +1183,17 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>toy</t>
+          <t>qa</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>qa</t>
+          <t>dataset</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1237,17 +1237,17 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>P127</t>
+          <t>beam</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>tokens</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1291,17 +1291,17 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>P159</t>
+          <t>beam</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>tokens</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1345,17 +1345,17 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>P20</t>
+          <t>beam</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>tokens</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">

</xml_diff>

<commit_message>
rel eval unified results
</commit_message>
<xml_diff>
--- a/results/reliability_eval/unified_scores_table.xlsx
+++ b/results/reliability_eval/unified_scores_table.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:O16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,20 +481,25 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>Dataset Name</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Beam Search</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Max New Tokens</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Temperature</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Strategy</t>
         </is>
@@ -535,22 +540,23 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>P178</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>temp_fact_statement</t>
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>10</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
         </is>
       </c>
     </row>
@@ -589,22 +595,23 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>P101</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>temp_fact_statement</t>
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
         </is>
       </c>
     </row>
@@ -643,22 +650,23 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>P1376</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>temp_fact_statement</t>
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>10</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
         </is>
       </c>
     </row>
@@ -697,22 +705,23 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>P103</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>temp_fact_statement</t>
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>10</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
         </is>
       </c>
     </row>
@@ -751,22 +760,23 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>P27</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>temp_fact_statement</t>
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>10</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
         </is>
       </c>
     </row>
@@ -805,22 +815,23 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>P108</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>temp_fact_statement</t>
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>10</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
         </is>
       </c>
     </row>
@@ -859,22 +870,23 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>temp_fact_statement</t>
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>10</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
         </is>
       </c>
     </row>
@@ -913,22 +925,23 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>P176</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>temp_fact_statement</t>
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>10</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
         </is>
       </c>
     </row>
@@ -967,22 +980,23 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>P19</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>temp_fact_statement</t>
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>10</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
         </is>
       </c>
     </row>
@@ -1021,22 +1035,23 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>P264</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>temp_fact_statement</t>
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>10</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
         </is>
       </c>
     </row>
@@ -1075,43 +1090,44 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>P1412</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>temp_fact_statement</t>
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="M12" t="n">
+        <v>10</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0.5993761140819964</v>
+        <v>0.975</v>
       </c>
       <c r="B13" t="n">
-        <v>0.7336791949116991</v>
+        <v>0.9930555555555556</v>
       </c>
       <c r="C13" t="n">
-        <v>0.5993761140819964</v>
+        <v>0.975</v>
       </c>
       <c r="D13" t="n">
-        <v>0.7336791949116991</v>
+        <v>0.9930555555555556</v>
       </c>
       <c r="E13" t="n">
-        <v>0.7210338680926915</v>
+        <v>0.225</v>
       </c>
       <c r="F13" t="n">
-        <v>0.7954849572290172</v>
+        <v>0.6500599549336971</v>
       </c>
       <c r="G13" t="n">
         <v>1</v>
@@ -1120,7 +1136,7 @@
         <v>1</v>
       </c>
       <c r="I13" t="n">
-        <v>0.66</v>
+        <v>0.7619047619047619</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -1129,20 +1145,21 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>toy-qa-dataset</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>tokens</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>temp</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="M13" t="n">
+        <v>10</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O13" t="inlineStr">
         <is>
           <t>fact_statement</t>
         </is>
@@ -1150,22 +1167,22 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0.975</v>
+        <v>0.4870766488413548</v>
       </c>
       <c r="B14" t="n">
-        <v>0.9930555555555556</v>
+        <v>0.6700312284531162</v>
       </c>
       <c r="C14" t="n">
-        <v>0.975</v>
+        <v>0.4870766488413548</v>
       </c>
       <c r="D14" t="n">
-        <v>0.9930555555555556</v>
+        <v>0.6700312284531162</v>
       </c>
       <c r="E14" t="n">
-        <v>0.225</v>
+        <v>0.7455436720142603</v>
       </c>
       <c r="F14" t="n">
-        <v>0.6500599549336971</v>
+        <v>0.8619193651115542</v>
       </c>
       <c r="G14" t="n">
         <v>1</v>
@@ -1174,7 +1191,7 @@
         <v>1</v>
       </c>
       <c r="I14" t="n">
-        <v>0.7619047619047619</v>
+        <v>0.66</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -1183,43 +1200,44 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>qa</t>
+          <t>P127</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>dataset</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>tokens_0.1_temp_fact_statement</t>
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="M14" t="n">
+        <v>10</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0.4870766488413548</v>
+        <v>0.5993761140819964</v>
       </c>
       <c r="B15" t="n">
-        <v>0.6700312284531162</v>
+        <v>0.7336791949116991</v>
       </c>
       <c r="C15" t="n">
-        <v>0.4870766488413548</v>
+        <v>0.5993761140819964</v>
       </c>
       <c r="D15" t="n">
-        <v>0.6700312284531162</v>
+        <v>0.7336791949116991</v>
       </c>
       <c r="E15" t="n">
-        <v>0.7455436720142603</v>
+        <v>0.7210338680926915</v>
       </c>
       <c r="F15" t="n">
-        <v>0.8619193651115542</v>
+        <v>0.7954849572290172</v>
       </c>
       <c r="G15" t="n">
         <v>1</v>
@@ -1237,43 +1255,44 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>P159</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>temp_fact_statement</t>
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="M15" t="n">
+        <v>10</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0.5993761140819964</v>
+        <v>0.3763586956521739</v>
       </c>
       <c r="B16" t="n">
-        <v>0.7336791949116991</v>
+        <v>0.07590362811828386</v>
       </c>
       <c r="C16" t="n">
-        <v>0.5993761140819964</v>
+        <v>0.3763586956521739</v>
       </c>
       <c r="D16" t="n">
-        <v>0.7336791949116991</v>
+        <v>0.07590362811828386</v>
       </c>
       <c r="E16" t="n">
-        <v>0.7210338680926915</v>
+        <v>0.8097826086956521</v>
       </c>
       <c r="F16" t="n">
-        <v>0.7954849572290172</v>
+        <v>0.3232831710772887</v>
       </c>
       <c r="G16" t="n">
         <v>1</v>
@@ -1282,7 +1301,7 @@
         <v>1</v>
       </c>
       <c r="I16" t="n">
-        <v>0.66</v>
+        <v>0.08</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -1291,76 +1310,23 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>P20</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>temp_fact_statement</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>0.3763586956521739</v>
-      </c>
-      <c r="B17" t="n">
-        <v>0.07590362811828386</v>
-      </c>
-      <c r="C17" t="n">
-        <v>0.3763586956521739</v>
-      </c>
-      <c r="D17" t="n">
-        <v>0.07590362811828386</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0.8097826086956521</v>
-      </c>
-      <c r="F17" t="n">
-        <v>0.3232831710772887</v>
-      </c>
-      <c r="G17" t="n">
-        <v>1</v>
-      </c>
-      <c r="H17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I17" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>Llama-3-8B</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>beam</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>temp_fact_statement</t>
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="M16" t="n">
+        <v>10</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
         </is>
       </c>
     </row>

</xml_diff>